<commit_message>
Distinguish calibrated and model spatial units
</commit_message>
<xml_diff>
--- a/SHOWCASE/paper_statistics.xlsx
+++ b/SHOWCASE/paper_statistics.xlsx
@@ -111,19 +111,19 @@
     <t>model units / worker</t>
   </si>
   <si>
-    <t>km^2</t>
-  </si>
-  <si>
-    <t>people / km^2</t>
-  </si>
-  <si>
-    <t>km</t>
-  </si>
-  <si>
-    <t>km^2 of floors</t>
-  </si>
-  <si>
-    <t>model units / m^2</t>
+    <t>model area units</t>
+  </si>
+  <si>
+    <t>people / model area unit</t>
+  </si>
+  <si>
+    <t>model distance units</t>
+  </si>
+  <si>
+    <t>model floor-space units</t>
+  </si>
+  <si>
+    <t>model monetary units / model floor-space unit</t>
   </si>
   <si>
     <t>index</t>
@@ -138,7 +138,7 @@
     <t>utility units</t>
   </si>
   <si>
-    <t>m^2 / resident</t>
+    <t>model floor-space units / resident</t>
   </si>
   <si>
     <t>%</t>
@@ -200,7 +200,7 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="44.42578125" customWidth="true"/>
-    <col min="2" max="2" width="20.85546875" customWidth="true"/>
+    <col min="2" max="2" width="42.5703125" customWidth="true"/>
     <col min="3" max="3" width="15.7109375" customWidth="true"/>
     <col min="4" max="4" width="15.7109375" customWidth="true"/>
     <col min="5" max="5" width="13.42578125" customWidth="true"/>
@@ -452,10 +452,10 @@
         <v>36</v>
       </c>
       <c r="C15" s="0">
-        <v>0.0004449378639393078</v>
+        <v>444.93786393930782</v>
       </c>
       <c r="D15" s="0">
-        <v>0.0004820837252557622</v>
+        <v>482.0837252557622</v>
       </c>
       <c r="E15" s="0">
         <v>8.3485502869050663</v>
@@ -469,13 +469,13 @@
         <v>36</v>
       </c>
       <c r="C16" s="0">
-        <v>0.00081149447093326315</v>
+        <v>811.49447093326319</v>
       </c>
       <c r="D16" s="0">
-        <v>0.00077196733133485737</v>
+        <v>771.96733133485736</v>
       </c>
       <c r="E16" s="0">
-        <v>-4.8709068286007406</v>
+        <v>-4.8709068286007522</v>
       </c>
     </row>
     <row r="17">
@@ -622,10 +622,10 @@
         <v>41</v>
       </c>
       <c r="C25" s="0">
-        <v>955.70796075314047</v>
+        <v>0.00095570796075314043</v>
       </c>
       <c r="D25" s="0">
-        <v>827.43743967859598</v>
+        <v>0.00082743743967859593</v>
       </c>
       <c r="E25" s="0">
         <v>-13.421518533073806</v>

</xml_diff>